<commit_message>
add v6.5 navlungo qa cargo integration gates
</commit_message>
<xml_diff>
--- a/02_SHEET_SISTEM/Tesbih_Kuyusu_V6_5_Ultra_Operasyon_Sheet.xlsx
+++ b/02_SHEET_SISTEM/Tesbih_Kuyusu_V6_5_Ultra_Operasyon_Sheet.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_WHATSAPP_KUYRUGU" sheetId="1" r:id="R84f13ced1df44544"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ACIK_SIPARISLER" sheetId="2" r:id="R20ced0f296114772"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_URUN_KALEMLERI" sheetId="3" r:id="R764a8f94596a4ca8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ODEMELER" sheetId="4" r:id="Rbdc7a5ba0d284f57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_FATURA_GRUPLARI" sheetId="5" r:id="Rb6f0eabdcdca4426"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_PARASUT_FATURA" sheetId="6" r:id="R5bed5a2220844973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_KARGO_PAKETLERI" sheetId="7" r:id="R0eef6208992643c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_MUSTERI_HAFIZA" sheetId="8" r:id="R6b7c98f51b5341d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_808_FINANS_ONIZLEME" sheetId="9" r:id="Rde4a8bc4248040ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_EBELGE_ISTISNA" sheetId="10" r:id="Rd5624a2cf2254096"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_KONTROL_MERKEZI" sheetId="11" r:id="R429caa3e21d9483b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_BANKA_HAREKETLERI" sheetId="12" r:id="R253bf61ad8954435"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_MUSTERI_ADRESLERI" sheetId="13" r:id="R04e07bc73fae4908"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_KULLANIM_KILAVUZU" sheetId="14" r:id="Ra842046f78b6483c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_AYARLAR" sheetId="15" r:id="Rc8874667f51b4039"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_VERI_SOZLUGU" sheetId="16" r:id="R0dee49dc310841b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_WHATSAPP_KUYRUGU" sheetId="1" r:id="R39f775ec0a2f497d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ACIK_SIPARISLER" sheetId="2" r:id="R0f2fa0e3c58b4e7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_URUN_KALEMLERI" sheetId="3" r:id="R696493272b8f4bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ODEMELER" sheetId="4" r:id="R08bab6b2d1d048ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_FATURA_GRUPLARI" sheetId="5" r:id="Rec6d4b1cff764182"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_PARASUT_FATURA" sheetId="6" r:id="Rda4270abc2d048a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_KARGO_PAKETLERI" sheetId="7" r:id="R123c4f64f662452b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_MUSTERI_HAFIZA" sheetId="8" r:id="Rf1a08fcb98fc45e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_808_FINANS_ONIZLEME" sheetId="9" r:id="Re8df2ba959a0447d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_EBELGE_ISTISNA" sheetId="10" r:id="R23eed220fc4243b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_KONTROL_MERKEZI" sheetId="11" r:id="Rb646dc7e20244b37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_BANKA_HAREKETLERI" sheetId="12" r:id="R5218de48827d45e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_MUSTERI_ADRESLERI" sheetId="13" r:id="R88f30dd4f2634645"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_KULLANIM_KILAVUZU" sheetId="14" r:id="R6e55b4eaf89c45f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_AYARLAR" sheetId="15" r:id="R2c7a89f051f54844"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_VERI_SOZLUGU" sheetId="16" r:id="R4369309b5b0a4ee3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4025,29 +4025,31 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>SISTEM_OPERASYON_SAATI_KAPANIS</x:v>
+        <x:v>NAVLUNGO_ENV</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>16:00</x:v>
+        <x:v>QA</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>Operasyon kapanış saati</x:v>
+        <x:v>Navlungo ortamı</x:v>
       </x:c>
       <x:c r="D9" t="str">
         <x:v>Evet</x:v>
       </x:c>
       <x:c r="E9" t="str"/>
-      <x:c r="F9" t="str"/>
+      <x:c r="F9" t="str">
+        <x:v>QA veya LIVE</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>TCKN_VARSAYILAN_GERCEK_KISI</x:v>
+        <x:v>NAVLUNGO_TEST_MODE</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>11111111111</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>Gerçek kişi TCKN boşsa uygulanabilir</x:v>
+        <x:v>İlk Navlungo testlerinde kontrollü alıcı kullanılır</x:v>
       </x:c>
       <x:c r="D10" t="str">
         <x:v>Evet</x:v>
@@ -4057,51 +4059,147 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>BANKA_HAREKET_MODULU_AKTIF</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>Evet</x:v>
-      </x:c>
+        <x:v>NAVLUNGO_SENDER_ADDRESS_ID</x:v>
+      </x:c>
+      <x:c r="B11" t="str"/>
       <x:c r="C11" t="str">
-        <x:v>14 banka hareketi teyit katmanı</x:v>
+        <x:v>Navlungo kayıtlı gönderici adres ID</x:v>
       </x:c>
       <x:c r="D11" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="E11" t="str"/>
-      <x:c r="F11" t="str"/>
+      <x:c r="F11" t="str">
+        <x:v>Script Properties önceliklidir</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>VARSAYILAN_KARGO_FIRMASI</x:v>
+        <x:v>NAVLUNGO_DEFAULT_CARRIER_ID</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Aras Kargo</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>Kargo firması önerisi</x:v>
+        <x:v>Varsayılan Navlungo taşıyıcı ID</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="E12" t="str"/>
       <x:c r="F12" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>KARGO_UCRETI_STANDART</x:v>
+        <x:v>NAVLUNGO_DEFAULT_POST_TYPE</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>125</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>808 finans ön izleme için varsayılan maliyet</x:v>
+        <x:v>Varsayılan Navlungo gönderi tipi</x:v>
       </x:c>
       <x:c r="D13" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="E13" t="str"/>
       <x:c r="F13" t="str"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>NAVLUNGO_DEFAULT_BARCODE_FORMAT</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Varsayılan Navlungo barkod formatı</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>Evet</x:v>
+      </x:c>
+      <x:c r="E14" t="str"/>
+      <x:c r="F14" t="str"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>SISTEM_OPERASYON_SAATI_KAPANIS</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>16:00</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Operasyon kapanış saati</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>Evet</x:v>
+      </x:c>
+      <x:c r="E15" t="str"/>
+      <x:c r="F15" t="str"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>TCKN_VARSAYILAN_GERCEK_KISI</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>11111111111</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Gerçek kişi TCKN boşsa uygulanabilir</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>Evet</x:v>
+      </x:c>
+      <x:c r="E16" t="str"/>
+      <x:c r="F16" t="str"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>BANKA_HAREKET_MODULU_AKTIF</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>Evet</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>14 banka hareketi teyit katmanı</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>Evet</x:v>
+      </x:c>
+      <x:c r="E17" t="str"/>
+      <x:c r="F17" t="str"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>VARSAYILAN_KARGO_FIRMASI</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>Aras Kargo</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>Kargo firması önerisi</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="E18" t="str"/>
+      <x:c r="F18" t="str"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>KARGO_UCRETI_STANDART</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>808 finans ön izleme için varsayılan maliyet</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="E19" t="str"/>
+      <x:c r="F19" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7257,16 +7355,16 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B158" t="str">
-        <x:v>Kontrol_Uyarısı</x:v>
+        <x:v>Navlungo_Gonderi_ID</x:v>
       </x:c>
       <x:c r="C158" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D158" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E158" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F158" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7274,19 +7372,19 @@
     </x:row>
     <x:row r="159">
       <x:c r="A159" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B159" t="str">
-        <x:v>WhatsApp_Tel</x:v>
+        <x:v>Navlungo_Barkod_No</x:v>
       </x:c>
       <x:c r="C159" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D159" t="str">
-        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E159" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F159" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7294,13 +7392,13 @@
     </x:row>
     <x:row r="160">
       <x:c r="A160" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B160" t="str">
-        <x:v>Sipariş_Sahibi</x:v>
+        <x:v>Navlungo_Takip_No</x:v>
       </x:c>
       <x:c r="C160" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D160" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
@@ -7314,16 +7412,16 @@
     </x:row>
     <x:row r="161">
       <x:c r="A161" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B161" t="str">
-        <x:v>Son_Kargo_Alıcısı</x:v>
+        <x:v>Navlungo_Etiket_URL</x:v>
       </x:c>
       <x:c r="C161" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D161" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E161" t="str">
         <x:v>Hayır</x:v>
@@ -7334,16 +7432,16 @@
     </x:row>
     <x:row r="162">
       <x:c r="A162" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B162" t="str">
-        <x:v>Son_Kargo_Tel</x:v>
+        <x:v>Navlungo_Durum</x:v>
       </x:c>
       <x:c r="C162" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D162" t="str">
-        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E162" t="str">
         <x:v>Evet</x:v>
@@ -7354,16 +7452,16 @@
     </x:row>
     <x:row r="163">
       <x:c r="A163" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B163" t="str">
-        <x:v>Son_İl</x:v>
+        <x:v>Navlungo_Hata_Mesaji</x:v>
       </x:c>
       <x:c r="C163" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D163" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E163" t="str">
         <x:v>Hayır</x:v>
@@ -7374,16 +7472,16 @@
     </x:row>
     <x:row r="164">
       <x:c r="A164" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B164" t="str">
-        <x:v>Son_İlçe</x:v>
+        <x:v>Navlungo_Payload_JSON</x:v>
       </x:c>
       <x:c r="C164" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D164" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E164" t="str">
         <x:v>Hayır</x:v>
@@ -7394,16 +7492,16 @@
     </x:row>
     <x:row r="165">
       <x:c r="A165" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B165" t="str">
-        <x:v>Son_Adres</x:v>
+        <x:v>Navlungo_Response_JSON</x:v>
       </x:c>
       <x:c r="C165" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D165" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E165" t="str">
         <x:v>Hayır</x:v>
@@ -7414,16 +7512,16 @@
     </x:row>
     <x:row r="166">
       <x:c r="A166" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B166" t="str">
-        <x:v>Son_Fatura_Kişisi</x:v>
+        <x:v>Test_Kargo_Mu</x:v>
       </x:c>
       <x:c r="C166" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D166" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E166" t="str">
         <x:v>Hayır</x:v>
@@ -7434,19 +7532,19 @@
     </x:row>
     <x:row r="167">
       <x:c r="A167" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B167" t="str">
-        <x:v>Son_Fatura_Tel</x:v>
+        <x:v>Navlungo_Olusturma_Tarihi</x:v>
       </x:c>
       <x:c r="C167" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D167" t="str">
-        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
+        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
       </x:c>
       <x:c r="E167" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F167" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7454,16 +7552,16 @@
     </x:row>
     <x:row r="168">
       <x:c r="A168" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B168" t="str">
-        <x:v>Son_Fatura_TCKN_VKN</x:v>
+        <x:v>Navlungo_Iptal_Tarihi</x:v>
       </x:c>
       <x:c r="C168" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D168" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
       </x:c>
       <x:c r="E168" t="str">
         <x:v>Hayır</x:v>
@@ -7474,19 +7572,19 @@
     </x:row>
     <x:row r="169">
       <x:c r="A169" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B169" t="str">
-        <x:v>Paraşüt_Cari_ID</x:v>
+        <x:v>Navlungo_Iptal_Sonucu</x:v>
       </x:c>
       <x:c r="C169" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D169" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E169" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F169" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7494,16 +7592,16 @@
     </x:row>
     <x:row r="170">
       <x:c r="A170" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B170" t="str">
-        <x:v>Son_Ödeme_Yapanlar_JSON</x:v>
+        <x:v>Kontrol_Uyarısı</x:v>
       </x:c>
       <x:c r="C170" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D170" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E170" t="str">
         <x:v>Hayır</x:v>
@@ -7517,16 +7615,16 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B171" t="str">
-        <x:v>Cari_Adaylari_JSON</x:v>
+        <x:v>WhatsApp_Tel</x:v>
       </x:c>
       <x:c r="C171" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D171" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
       </x:c>
       <x:c r="E171" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F171" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7537,13 +7635,13 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B172" t="str">
-        <x:v>Son_Kargo_Bilgisi_JSON</x:v>
+        <x:v>Sipariş_Sahibi</x:v>
       </x:c>
       <x:c r="C172" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D172" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E172" t="str">
         <x:v>Hayır</x:v>
@@ -7557,13 +7655,13 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B173" t="str">
-        <x:v>Güven_Puanı</x:v>
+        <x:v>Son_Kargo_Alıcısı</x:v>
       </x:c>
       <x:c r="C173" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D173" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E173" t="str">
         <x:v>Hayır</x:v>
@@ -7577,13 +7675,13 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B174" t="str">
-        <x:v>Son_Başarılı_Sipariş_ID</x:v>
+        <x:v>Son_Kargo_Tel</x:v>
       </x:c>
       <x:c r="C174" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D174" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
       </x:c>
       <x:c r="E174" t="str">
         <x:v>Evet</x:v>
@@ -7597,13 +7695,13 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B175" t="str">
-        <x:v>Son_Güncelleme</x:v>
+        <x:v>Son_İl</x:v>
       </x:c>
       <x:c r="C175" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D175" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E175" t="str">
         <x:v>Hayır</x:v>
@@ -7617,13 +7715,13 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B176" t="str">
-        <x:v>Güven_Notu</x:v>
+        <x:v>Son_İlçe</x:v>
       </x:c>
       <x:c r="C176" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D176" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E176" t="str">
         <x:v>Hayır</x:v>
@@ -7637,13 +7735,13 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B177" t="str">
-        <x:v>Kontrol_Uyarısı</x:v>
+        <x:v>Son_Adres</x:v>
       </x:c>
       <x:c r="C177" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D177" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E177" t="str">
         <x:v>Hayır</x:v>
@@ -7654,19 +7752,19 @@
     </x:row>
     <x:row r="178">
       <x:c r="A178" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B178" t="str">
-        <x:v>808_Kayıt_ID</x:v>
+        <x:v>Son_Fatura_Kişisi</x:v>
       </x:c>
       <x:c r="C178" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D178" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E178" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F178" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7674,16 +7772,16 @@
     </x:row>
     <x:row r="179">
       <x:c r="A179" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B179" t="str">
-        <x:v>Açık_Sipariş_ID</x:v>
+        <x:v>Son_Fatura_Tel</x:v>
       </x:c>
       <x:c r="C179" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D179" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
       </x:c>
       <x:c r="E179" t="str">
         <x:v>Evet</x:v>
@@ -7694,16 +7792,16 @@
     </x:row>
     <x:row r="180">
       <x:c r="A180" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B180" t="str">
-        <x:v>Model_Tipi</x:v>
+        <x:v>Son_Fatura_TCKN_VKN</x:v>
       </x:c>
       <x:c r="C180" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D180" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E180" t="str">
         <x:v>Hayır</x:v>
@@ -7714,19 +7812,19 @@
     </x:row>
     <x:row r="181">
       <x:c r="A181" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B181" t="str">
-        <x:v>Ürün_Toplamı</x:v>
+        <x:v>Paraşüt_Cari_ID</x:v>
       </x:c>
       <x:c r="C181" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D181" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E181" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F181" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7734,16 +7832,16 @@
     </x:row>
     <x:row r="182">
       <x:c r="A182" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B182" t="str">
-        <x:v>KDV_Hariç</x:v>
+        <x:v>Son_Ödeme_Yapanlar_JSON</x:v>
       </x:c>
       <x:c r="C182" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D182" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E182" t="str">
         <x:v>Hayır</x:v>
@@ -7754,19 +7852,19 @@
     </x:row>
     <x:row r="183">
       <x:c r="A183" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B183" t="str">
-        <x:v>KDV_Tutarı</x:v>
+        <x:v>Cari_Adaylari_JSON</x:v>
       </x:c>
       <x:c r="C183" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D183" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E183" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F183" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7774,16 +7872,16 @@
     </x:row>
     <x:row r="184">
       <x:c r="A184" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B184" t="str">
-        <x:v>Ödeme_Toplamı</x:v>
+        <x:v>Son_Kargo_Bilgisi_JSON</x:v>
       </x:c>
       <x:c r="C184" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D184" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E184" t="str">
         <x:v>Hayır</x:v>
@@ -7794,13 +7892,13 @@
     </x:row>
     <x:row r="185">
       <x:c r="A185" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B185" t="str">
-        <x:v>Fark</x:v>
+        <x:v>Güven_Puanı</x:v>
       </x:c>
       <x:c r="C185" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D185" t="str">
         <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
@@ -7814,19 +7912,19 @@
     </x:row>
     <x:row r="186">
       <x:c r="A186" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B186" t="str">
-        <x:v>Net_Ticari_Kazanç</x:v>
+        <x:v>Son_Başarılı_Sipariş_ID</x:v>
       </x:c>
       <x:c r="C186" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D186" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E186" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F186" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7834,16 +7932,16 @@
     </x:row>
     <x:row r="187">
       <x:c r="A187" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B187" t="str">
-        <x:v>Resmi_Fatura_Notu</x:v>
+        <x:v>Son_Güncelleme</x:v>
       </x:c>
       <x:c r="C187" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D187" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E187" t="str">
         <x:v>Hayır</x:v>
@@ -7854,16 +7952,16 @@
     </x:row>
     <x:row r="188">
       <x:c r="A188" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B188" t="str">
-        <x:v>Fatura_Etkisi_Yok</x:v>
+        <x:v>Güven_Notu</x:v>
       </x:c>
       <x:c r="C188" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D188" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E188" t="str">
         <x:v>Hayır</x:v>
@@ -7874,13 +7972,13 @@
     </x:row>
     <x:row r="189">
       <x:c r="A189" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B189" t="str">
         <x:v>Kontrol_Uyarısı</x:v>
       </x:c>
       <x:c r="C189" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D189" t="str">
         <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
@@ -7894,13 +7992,13 @@
     </x:row>
     <x:row r="190">
       <x:c r="A190" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B190" t="str">
-        <x:v>E_Belge_Kayıt_ID</x:v>
+        <x:v>808_Kayıt_ID</x:v>
       </x:c>
       <x:c r="C190" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D190" t="str">
         <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
@@ -7914,13 +8012,13 @@
     </x:row>
     <x:row r="191">
       <x:c r="A191" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B191" t="str">
-        <x:v>Fatura_Grubu_ID</x:v>
+        <x:v>Açık_Sipariş_ID</x:v>
       </x:c>
       <x:c r="C191" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D191" t="str">
         <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
@@ -7934,19 +8032,19 @@
     </x:row>
     <x:row r="192">
       <x:c r="A192" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B192" t="str">
-        <x:v>Açık_Sipariş_ID</x:v>
+        <x:v>Model_Tipi</x:v>
       </x:c>
       <x:c r="C192" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D192" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E192" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F192" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7954,19 +8052,19 @@
     </x:row>
     <x:row r="193">
       <x:c r="A193" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B193" t="str">
-        <x:v>Paraşüt_Fatura_ID</x:v>
+        <x:v>Ürün_Toplamı</x:v>
       </x:c>
       <x:c r="C193" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D193" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E193" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F193" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7974,16 +8072,16 @@
     </x:row>
     <x:row r="194">
       <x:c r="A194" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B194" t="str">
-        <x:v>Fatura_Kişisi</x:v>
+        <x:v>KDV_Hariç</x:v>
       </x:c>
       <x:c r="C194" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D194" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E194" t="str">
         <x:v>Hayır</x:v>
@@ -7994,19 +8092,19 @@
     </x:row>
     <x:row r="195">
       <x:c r="A195" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B195" t="str">
-        <x:v>Fatura_TCKN_VKN</x:v>
+        <x:v>KDV_Tutarı</x:v>
       </x:c>
       <x:c r="C195" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D195" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E195" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F195" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8014,16 +8112,16 @@
     </x:row>
     <x:row r="196">
       <x:c r="A196" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B196" t="str">
-        <x:v>Cari_Tipi</x:v>
+        <x:v>Ödeme_Toplamı</x:v>
       </x:c>
       <x:c r="C196" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D196" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E196" t="str">
         <x:v>Hayır</x:v>
@@ -8034,16 +8132,16 @@
     </x:row>
     <x:row r="197">
       <x:c r="A197" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B197" t="str">
-        <x:v>E_Belge_Tipi</x:v>
+        <x:v>Fark</x:v>
       </x:c>
       <x:c r="C197" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D197" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E197" t="str">
         <x:v>Hayır</x:v>
@@ -8054,13 +8152,13 @@
     </x:row>
     <x:row r="198">
       <x:c r="A198" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B198" t="str">
-        <x:v>Gümüş_İçeriyor_Mu</x:v>
+        <x:v>Net_Ticari_Kazanç</x:v>
       </x:c>
       <x:c r="C198" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D198" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
@@ -8074,16 +8172,16 @@
     </x:row>
     <x:row r="199">
       <x:c r="A199" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B199" t="str">
-        <x:v>KDV0_Satırı_Var_Mı</x:v>
+        <x:v>Resmi_Fatura_Notu</x:v>
       </x:c>
       <x:c r="C199" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D199" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E199" t="str">
         <x:v>Hayır</x:v>
@@ -8094,16 +8192,16 @@
     </x:row>
     <x:row r="200">
       <x:c r="A200" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B200" t="str">
-        <x:v>İstisna_Gerekli_Mi</x:v>
+        <x:v>Fatura_Etkisi_Yok</x:v>
       </x:c>
       <x:c r="C200" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D200" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E200" t="str">
         <x:v>Hayır</x:v>
@@ -8114,19 +8212,19 @@
     </x:row>
     <x:row r="201">
       <x:c r="A201" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B201" t="str">
-        <x:v>İstisna_Kodu</x:v>
+        <x:v>Kontrol_Uyarısı</x:v>
       </x:c>
       <x:c r="C201" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D201" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E201" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F201" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8137,16 +8235,16 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B202" t="str">
-        <x:v>İstisna_Açıklama</x:v>
+        <x:v>E_Belge_Kayıt_ID</x:v>
       </x:c>
       <x:c r="C202" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D202" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E202" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F202" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8157,13 +8255,13 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B203" t="str">
-        <x:v>Gönderim_Durumu</x:v>
+        <x:v>Fatura_Grubu_ID</x:v>
       </x:c>
       <x:c r="C203" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D203" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E203" t="str">
         <x:v>Evet</x:v>
@@ -8177,16 +8275,16 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B204" t="str">
-        <x:v>Resmi_Gönderim_Onayı</x:v>
+        <x:v>Açık_Sipariş_ID</x:v>
       </x:c>
       <x:c r="C204" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D204" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E204" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F204" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8197,16 +8295,16 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B205" t="str">
-        <x:v>Resmi_Gönderim_Blokaj_Nedeni</x:v>
+        <x:v>Paraşüt_Fatura_ID</x:v>
       </x:c>
       <x:c r="C205" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D205" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E205" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F205" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8217,13 +8315,13 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B206" t="str">
-        <x:v>Kontrol_Seviyesi</x:v>
+        <x:v>Fatura_Kişisi</x:v>
       </x:c>
       <x:c r="C206" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D206" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E206" t="str">
         <x:v>Hayır</x:v>
@@ -8234,19 +8332,19 @@
     </x:row>
     <x:row r="207">
       <x:c r="A207" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B207" t="str">
-        <x:v>Kontrol_ID</x:v>
+        <x:v>Fatura_TCKN_VKN</x:v>
       </x:c>
       <x:c r="C207" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D207" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E207" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F207" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8254,16 +8352,16 @@
     </x:row>
     <x:row r="208">
       <x:c r="A208" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B208" t="str">
-        <x:v>Tarih</x:v>
+        <x:v>Cari_Tipi</x:v>
       </x:c>
       <x:c r="C208" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D208" t="str">
-        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E208" t="str">
         <x:v>Hayır</x:v>
@@ -8274,13 +8372,13 @@
     </x:row>
     <x:row r="209">
       <x:c r="A209" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B209" t="str">
-        <x:v>Kaynak_Sayfa</x:v>
+        <x:v>E_Belge_Tipi</x:v>
       </x:c>
       <x:c r="C209" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D209" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
@@ -8294,19 +8392,19 @@
     </x:row>
     <x:row r="210">
       <x:c r="A210" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B210" t="str">
-        <x:v>Kaynak_ID</x:v>
+        <x:v>Gümüş_İçeriyor_Mu</x:v>
       </x:c>
       <x:c r="C210" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D210" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E210" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F210" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8314,16 +8412,16 @@
     </x:row>
     <x:row r="211">
       <x:c r="A211" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B211" t="str">
-        <x:v>Kontrol_Tipi</x:v>
+        <x:v>KDV0_Satırı_Var_Mı</x:v>
       </x:c>
       <x:c r="C211" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D211" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E211" t="str">
         <x:v>Hayır</x:v>
@@ -8334,13 +8432,13 @@
     </x:row>
     <x:row r="212">
       <x:c r="A212" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B212" t="str">
-        <x:v>Risk_Seviyesi</x:v>
+        <x:v>İstisna_Gerekli_Mi</x:v>
       </x:c>
       <x:c r="C212" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D212" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
@@ -8354,16 +8452,16 @@
     </x:row>
     <x:row r="213">
       <x:c r="A213" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B213" t="str">
-        <x:v>Durum</x:v>
+        <x:v>İstisna_Kodu</x:v>
       </x:c>
       <x:c r="C213" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D213" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E213" t="str">
         <x:v>Evet</x:v>
@@ -8374,13 +8472,13 @@
     </x:row>
     <x:row r="214">
       <x:c r="A214" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B214" t="str">
-        <x:v>Kontrol_Uyarısı</x:v>
+        <x:v>İstisna_Açıklama</x:v>
       </x:c>
       <x:c r="C214" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D214" t="str">
         <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
@@ -8394,19 +8492,19 @@
     </x:row>
     <x:row r="215">
       <x:c r="A215" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B215" t="str">
-        <x:v>Beklenen_Aksiyon</x:v>
+        <x:v>Gönderim_Durumu</x:v>
       </x:c>
       <x:c r="C215" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D215" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E215" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F215" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8414,16 +8512,16 @@
     </x:row>
     <x:row r="216">
       <x:c r="A216" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B216" t="str">
-        <x:v>Sorumlu</x:v>
+        <x:v>Resmi_Gönderim_Onayı</x:v>
       </x:c>
       <x:c r="C216" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D216" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E216" t="str">
         <x:v>Hayır</x:v>
@@ -8434,16 +8532,16 @@
     </x:row>
     <x:row r="217">
       <x:c r="A217" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B217" t="str">
-        <x:v>Çözüm_Notu</x:v>
+        <x:v>Resmi_Gönderim_Blokaj_Nedeni</x:v>
       </x:c>
       <x:c r="C217" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D217" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E217" t="str">
         <x:v>Hayır</x:v>
@@ -8454,16 +8552,16 @@
     </x:row>
     <x:row r="218">
       <x:c r="A218" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B218" t="str">
-        <x:v>Kapanış_Tarihi</x:v>
+        <x:v>Kontrol_Seviyesi</x:v>
       </x:c>
       <x:c r="C218" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D218" t="str">
-        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E218" t="str">
         <x:v>Hayır</x:v>
@@ -8477,16 +8575,16 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B219" t="str">
-        <x:v>Blokaj_Mı</x:v>
+        <x:v>Kontrol_ID</x:v>
       </x:c>
       <x:c r="C219" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D219" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E219" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F219" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8497,13 +8595,13 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B220" t="str">
-        <x:v>İlgili_Modül</x:v>
+        <x:v>Tarih</x:v>
       </x:c>
       <x:c r="C220" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D220" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
       </x:c>
       <x:c r="E220" t="str">
         <x:v>Hayır</x:v>
@@ -8514,16 +8612,16 @@
     </x:row>
     <x:row r="221">
       <x:c r="A221" t="str">
-        <x:v>13_VERI_SOZLUGU</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B221" t="str">
-        <x:v>Sayfa</x:v>
+        <x:v>Kaynak_Sayfa</x:v>
       </x:c>
       <x:c r="C221" t="str">
-        <x:v>Koddan üretilen kolon sözlüğü</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D221" t="str">
-        <x:v>Veri sözlüğü alanını tanımlamak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E221" t="str">
         <x:v>Hayır</x:v>
@@ -8534,19 +8632,19 @@
     </x:row>
     <x:row r="222">
       <x:c r="A222" t="str">
-        <x:v>13_VERI_SOZLUGU</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B222" t="str">
-        <x:v>Kolon</x:v>
+        <x:v>Kaynak_ID</x:v>
       </x:c>
       <x:c r="C222" t="str">
-        <x:v>Koddan üretilen kolon sözlüğü</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D222" t="str">
-        <x:v>Veri sözlüğü alanını tanımlamak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E222" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F222" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8554,16 +8652,16 @@
     </x:row>
     <x:row r="223">
       <x:c r="A223" t="str">
-        <x:v>13_VERI_SOZLUGU</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B223" t="str">
-        <x:v>Kaynak</x:v>
+        <x:v>Kontrol_Tipi</x:v>
       </x:c>
       <x:c r="C223" t="str">
-        <x:v>Koddan üretilen kolon sözlüğü</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D223" t="str">
-        <x:v>Veri sözlüğü alanını tanımlamak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E223" t="str">
         <x:v>Hayır</x:v>
@@ -8574,16 +8672,16 @@
     </x:row>
     <x:row r="224">
       <x:c r="A224" t="str">
-        <x:v>13_VERI_SOZLUGU</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B224" t="str">
-        <x:v>Amaç</x:v>
+        <x:v>Risk_Seviyesi</x:v>
       </x:c>
       <x:c r="C224" t="str">
-        <x:v>Koddan üretilen kolon sözlüğü</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D224" t="str">
-        <x:v>Veri sözlüğü alanını tanımlamak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E224" t="str">
         <x:v>Hayır</x:v>
@@ -8594,19 +8692,19 @@
     </x:row>
     <x:row r="225">
       <x:c r="A225" t="str">
-        <x:v>13_VERI_SOZLUGU</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B225" t="str">
-        <x:v>Zorunlu_Mu</x:v>
+        <x:v>Durum</x:v>
       </x:c>
       <x:c r="C225" t="str">
-        <x:v>Koddan üretilen kolon sözlüğü</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D225" t="str">
-        <x:v>Veri sözlüğü alanını tanımlamak</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E225" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F225" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8614,13 +8712,13 @@
     </x:row>
     <x:row r="226">
       <x:c r="A226" t="str">
-        <x:v>13_VERI_SOZLUGU</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B226" t="str">
-        <x:v>Not</x:v>
+        <x:v>Kontrol_Uyarısı</x:v>
       </x:c>
       <x:c r="C226" t="str">
-        <x:v>Koddan üretilen kolon sözlüğü</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D226" t="str">
         <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
@@ -8634,19 +8732,19 @@
     </x:row>
     <x:row r="227">
       <x:c r="A227" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B227" t="str">
-        <x:v>Banka_Hareket_ID</x:v>
+        <x:v>Beklenen_Aksiyon</x:v>
       </x:c>
       <x:c r="C227" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D227" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E227" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F227" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8654,16 +8752,16 @@
     </x:row>
     <x:row r="228">
       <x:c r="A228" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B228" t="str">
-        <x:v>İşlem_Tarihi</x:v>
+        <x:v>Sorumlu</x:v>
       </x:c>
       <x:c r="C228" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D228" t="str">
-        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E228" t="str">
         <x:v>Hayır</x:v>
@@ -8674,16 +8772,16 @@
     </x:row>
     <x:row r="229">
       <x:c r="A229" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B229" t="str">
-        <x:v>Valör_Tarihi</x:v>
+        <x:v>Çözüm_Notu</x:v>
       </x:c>
       <x:c r="C229" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D229" t="str">
-        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E229" t="str">
         <x:v>Hayır</x:v>
@@ -8694,19 +8792,19 @@
     </x:row>
     <x:row r="230">
       <x:c r="A230" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B230" t="str">
-        <x:v>Gönderen_Adı</x:v>
+        <x:v>Kapanış_Tarihi</x:v>
       </x:c>
       <x:c r="C230" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D230" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
       </x:c>
       <x:c r="E230" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F230" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8714,16 +8812,16 @@
     </x:row>
     <x:row r="231">
       <x:c r="A231" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B231" t="str">
-        <x:v>Açıklama</x:v>
+        <x:v>Blokaj_Mı</x:v>
       </x:c>
       <x:c r="C231" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D231" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E231" t="str">
         <x:v>Hayır</x:v>
@@ -8734,19 +8832,19 @@
     </x:row>
     <x:row r="232">
       <x:c r="A232" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B232" t="str">
-        <x:v>Tutar</x:v>
+        <x:v>İlgili_Modül</x:v>
       </x:c>
       <x:c r="C232" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D232" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E232" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F232" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8754,19 +8852,19 @@
     </x:row>
     <x:row r="233">
       <x:c r="A233" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>13_VERI_SOZLUGU</x:v>
       </x:c>
       <x:c r="B233" t="str">
-        <x:v>Banka_Adı</x:v>
+        <x:v>Sayfa</x:v>
       </x:c>
       <x:c r="C233" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Koddan üretilen kolon sözlüğü</x:v>
       </x:c>
       <x:c r="D233" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Veri sözlüğü alanını tanımlamak</x:v>
       </x:c>
       <x:c r="E233" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F233" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8774,16 +8872,16 @@
     </x:row>
     <x:row r="234">
       <x:c r="A234" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>13_VERI_SOZLUGU</x:v>
       </x:c>
       <x:c r="B234" t="str">
-        <x:v>IBAN</x:v>
+        <x:v>Kolon</x:v>
       </x:c>
       <x:c r="C234" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Koddan üretilen kolon sözlüğü</x:v>
       </x:c>
       <x:c r="D234" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Veri sözlüğü alanını tanımlamak</x:v>
       </x:c>
       <x:c r="E234" t="str">
         <x:v>Hayır</x:v>
@@ -8794,16 +8892,16 @@
     </x:row>
     <x:row r="235">
       <x:c r="A235" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>13_VERI_SOZLUGU</x:v>
       </x:c>
       <x:c r="B235" t="str">
-        <x:v>İşlem_Tipi</x:v>
+        <x:v>Kaynak</x:v>
       </x:c>
       <x:c r="C235" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Koddan üretilen kolon sözlüğü</x:v>
       </x:c>
       <x:c r="D235" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Veri sözlüğü alanını tanımlamak</x:v>
       </x:c>
       <x:c r="E235" t="str">
         <x:v>Hayır</x:v>
@@ -8814,16 +8912,16 @@
     </x:row>
     <x:row r="236">
       <x:c r="A236" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>13_VERI_SOZLUGU</x:v>
       </x:c>
       <x:c r="B236" t="str">
-        <x:v>Referans_No</x:v>
+        <x:v>Amaç</x:v>
       </x:c>
       <x:c r="C236" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Koddan üretilen kolon sözlüğü</x:v>
       </x:c>
       <x:c r="D236" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Veri sözlüğü alanını tanımlamak</x:v>
       </x:c>
       <x:c r="E236" t="str">
         <x:v>Hayır</x:v>
@@ -8834,19 +8932,19 @@
     </x:row>
     <x:row r="237">
       <x:c r="A237" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>13_VERI_SOZLUGU</x:v>
       </x:c>
       <x:c r="B237" t="str">
-        <x:v>Eşleşme_Durumu</x:v>
+        <x:v>Zorunlu_Mu</x:v>
       </x:c>
       <x:c r="C237" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Koddan üretilen kolon sözlüğü</x:v>
       </x:c>
       <x:c r="D237" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>Veri sözlüğü alanını tanımlamak</x:v>
       </x:c>
       <x:c r="E237" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F237" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8854,16 +8952,16 @@
     </x:row>
     <x:row r="238">
       <x:c r="A238" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>13_VERI_SOZLUGU</x:v>
       </x:c>
       <x:c r="B238" t="str">
-        <x:v>Eşleşme_Puanı</x:v>
+        <x:v>Not</x:v>
       </x:c>
       <x:c r="C238" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Koddan üretilen kolon sözlüğü</x:v>
       </x:c>
       <x:c r="D238" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E238" t="str">
         <x:v>Hayır</x:v>
@@ -8877,7 +8975,7 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B239" t="str">
-        <x:v>Önerilen_Açık_Sipariş_ID</x:v>
+        <x:v>Banka_Hareket_ID</x:v>
       </x:c>
       <x:c r="C239" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
@@ -8897,16 +8995,16 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B240" t="str">
-        <x:v>Önerilen_Ödeme_ID</x:v>
+        <x:v>İşlem_Tarihi</x:v>
       </x:c>
       <x:c r="C240" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D240" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
       </x:c>
       <x:c r="E240" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F240" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8917,13 +9015,13 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B241" t="str">
-        <x:v>Önerilen_Ödeme_Yapan</x:v>
+        <x:v>Valör_Tarihi</x:v>
       </x:c>
       <x:c r="C241" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D241" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
       </x:c>
       <x:c r="E241" t="str">
         <x:v>Hayır</x:v>
@@ -8937,16 +9035,16 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B242" t="str">
-        <x:v>Operatör_Onayı</x:v>
+        <x:v>Gönderen_Adı</x:v>
       </x:c>
       <x:c r="C242" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D242" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E242" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F242" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8957,7 +9055,7 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B243" t="str">
-        <x:v>Kontrol_Uyarısı</x:v>
+        <x:v>Açıklama</x:v>
       </x:c>
       <x:c r="C243" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
@@ -8974,16 +9072,16 @@
     </x:row>
     <x:row r="244">
       <x:c r="A244" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B244" t="str">
-        <x:v>Adres_ID</x:v>
+        <x:v>Tutar</x:v>
       </x:c>
       <x:c r="C244" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D244" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E244" t="str">
         <x:v>Evet</x:v>
@@ -8994,16 +9092,16 @@
     </x:row>
     <x:row r="245">
       <x:c r="A245" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B245" t="str">
-        <x:v>WhatsApp_Tel</x:v>
+        <x:v>Banka_Adı</x:v>
       </x:c>
       <x:c r="C245" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D245" t="str">
-        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E245" t="str">
         <x:v>Evet</x:v>
@@ -9014,13 +9112,13 @@
     </x:row>
     <x:row r="246">
       <x:c r="A246" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B246" t="str">
-        <x:v>Sipariş_Sahibi</x:v>
+        <x:v>IBAN</x:v>
       </x:c>
       <x:c r="C246" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D246" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
@@ -9034,16 +9132,16 @@
     </x:row>
     <x:row r="247">
       <x:c r="A247" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B247" t="str">
-        <x:v>Kargo_Alıcısı</x:v>
+        <x:v>İşlem_Tipi</x:v>
       </x:c>
       <x:c r="C247" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D247" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E247" t="str">
         <x:v>Hayır</x:v>
@@ -9054,19 +9152,19 @@
     </x:row>
     <x:row r="248">
       <x:c r="A248" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B248" t="str">
-        <x:v>Kargo_Tel</x:v>
+        <x:v>Referans_No</x:v>
       </x:c>
       <x:c r="C248" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D248" t="str">
-        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E248" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F248" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9074,19 +9172,19 @@
     </x:row>
     <x:row r="249">
       <x:c r="A249" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B249" t="str">
-        <x:v>İl</x:v>
+        <x:v>Eşleşme_Durumu</x:v>
       </x:c>
       <x:c r="C249" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D249" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E249" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F249" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9094,16 +9192,16 @@
     </x:row>
     <x:row r="250">
       <x:c r="A250" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B250" t="str">
-        <x:v>İlçe</x:v>
+        <x:v>Eşleşme_Puanı</x:v>
       </x:c>
       <x:c r="C250" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D250" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E250" t="str">
         <x:v>Hayır</x:v>
@@ -9114,19 +9212,19 @@
     </x:row>
     <x:row r="251">
       <x:c r="A251" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B251" t="str">
-        <x:v>Adres</x:v>
+        <x:v>Önerilen_Açık_Sipariş_ID</x:v>
       </x:c>
       <x:c r="C251" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D251" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E251" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F251" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9134,19 +9232,19 @@
     </x:row>
     <x:row r="252">
       <x:c r="A252" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B252" t="str">
-        <x:v>Kargo_Firması</x:v>
+        <x:v>Önerilen_Ödeme_ID</x:v>
       </x:c>
       <x:c r="C252" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D252" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E252" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F252" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9154,13 +9252,13 @@
     </x:row>
     <x:row r="253">
       <x:c r="A253" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B253" t="str">
-        <x:v>Varsayılan_Mı</x:v>
+        <x:v>Önerilen_Ödeme_Yapan</x:v>
       </x:c>
       <x:c r="C253" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D253" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
@@ -9174,16 +9272,16 @@
     </x:row>
     <x:row r="254">
       <x:c r="A254" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B254" t="str">
-        <x:v>Son_Kullanım</x:v>
+        <x:v>Operatör_Onayı</x:v>
       </x:c>
       <x:c r="C254" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D254" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E254" t="str">
         <x:v>Hayır</x:v>
@@ -9194,19 +9292,19 @@
     </x:row>
     <x:row r="255">
       <x:c r="A255" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B255" t="str">
-        <x:v>Adres_Durumu</x:v>
+        <x:v>Kontrol_Uyarısı</x:v>
       </x:c>
       <x:c r="C255" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D255" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E255" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F255" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9217,18 +9315,258 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B256" t="str">
-        <x:v>Kontrol_Uyarısı</x:v>
+        <x:v>Adres_ID</x:v>
       </x:c>
       <x:c r="C256" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D256" t="str">
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+      </x:c>
+      <x:c r="E256" t="str">
+        <x:v>Evet</x:v>
+      </x:c>
+      <x:c r="F256" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="257">
+      <x:c r="A257" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B257" t="str">
+        <x:v>WhatsApp_Tel</x:v>
+      </x:c>
+      <x:c r="C257" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D257" t="str">
+        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
+      </x:c>
+      <x:c r="E257" t="str">
+        <x:v>Evet</x:v>
+      </x:c>
+      <x:c r="F257" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="258">
+      <x:c r="A258" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B258" t="str">
+        <x:v>Sipariş_Sahibi</x:v>
+      </x:c>
+      <x:c r="C258" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D258" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+      </x:c>
+      <x:c r="E258" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="F258" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259">
+      <x:c r="A259" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B259" t="str">
+        <x:v>Kargo_Alıcısı</x:v>
+      </x:c>
+      <x:c r="C259" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D259" t="str">
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+      </x:c>
+      <x:c r="E259" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="F259" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="260">
+      <x:c r="A260" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B260" t="str">
+        <x:v>Kargo_Tel</x:v>
+      </x:c>
+      <x:c r="C260" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D260" t="str">
+        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
+      </x:c>
+      <x:c r="E260" t="str">
+        <x:v>Evet</x:v>
+      </x:c>
+      <x:c r="F260" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="261">
+      <x:c r="A261" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B261" t="str">
+        <x:v>İl</x:v>
+      </x:c>
+      <x:c r="C261" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D261" t="str">
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+      </x:c>
+      <x:c r="E261" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="F261" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="262">
+      <x:c r="A262" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B262" t="str">
+        <x:v>İlçe</x:v>
+      </x:c>
+      <x:c r="C262" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D262" t="str">
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+      </x:c>
+      <x:c r="E262" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="F262" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="263">
+      <x:c r="A263" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B263" t="str">
+        <x:v>Adres</x:v>
+      </x:c>
+      <x:c r="C263" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D263" t="str">
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+      </x:c>
+      <x:c r="E263" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="F263" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="264">
+      <x:c r="A264" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B264" t="str">
+        <x:v>Kargo_Firması</x:v>
+      </x:c>
+      <x:c r="C264" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D264" t="str">
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+      </x:c>
+      <x:c r="E264" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="F264" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="265">
+      <x:c r="A265" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B265" t="str">
+        <x:v>Varsayılan_Mı</x:v>
+      </x:c>
+      <x:c r="C265" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D265" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+      </x:c>
+      <x:c r="E265" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="F265" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266">
+      <x:c r="A266" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B266" t="str">
+        <x:v>Son_Kullanım</x:v>
+      </x:c>
+      <x:c r="C266" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D266" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+      </x:c>
+      <x:c r="E266" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="F266" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267">
+      <x:c r="A267" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B267" t="str">
+        <x:v>Adres_Durumu</x:v>
+      </x:c>
+      <x:c r="C267" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D267" t="str">
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+      </x:c>
+      <x:c r="E267" t="str">
+        <x:v>Evet</x:v>
+      </x:c>
+      <x:c r="F267" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="268">
+      <x:c r="A268" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B268" t="str">
+        <x:v>Kontrol_Uyarısı</x:v>
+      </x:c>
+      <x:c r="C268" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D268" t="str">
         <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
-      <x:c r="E256" t="str">
-        <x:v>Hayır</x:v>
-      </x:c>
-      <x:c r="F256" t="str">
+      <x:c r="E268" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="F268" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
       </x:c>
     </x:row>
@@ -14860,6 +15198,42 @@
         <x:v>Paket_Notu</x:v>
       </x:c>
       <x:c r="N1" s="13" t="str">
+        <x:v>Navlungo_Gonderi_ID</x:v>
+      </x:c>
+      <x:c r="O1" t="str">
+        <x:v>Navlungo_Barkod_No</x:v>
+      </x:c>
+      <x:c r="P1" t="str">
+        <x:v>Navlungo_Takip_No</x:v>
+      </x:c>
+      <x:c r="Q1" t="str">
+        <x:v>Navlungo_Etiket_URL</x:v>
+      </x:c>
+      <x:c r="R1" t="str">
+        <x:v>Navlungo_Durum</x:v>
+      </x:c>
+      <x:c r="S1" t="str">
+        <x:v>Navlungo_Hata_Mesaji</x:v>
+      </x:c>
+      <x:c r="T1" t="str">
+        <x:v>Navlungo_Payload_JSON</x:v>
+      </x:c>
+      <x:c r="U1" t="str">
+        <x:v>Navlungo_Response_JSON</x:v>
+      </x:c>
+      <x:c r="V1" t="str">
+        <x:v>Test_Kargo_Mu</x:v>
+      </x:c>
+      <x:c r="W1" t="str">
+        <x:v>Navlungo_Olusturma_Tarihi</x:v>
+      </x:c>
+      <x:c r="X1" t="str">
+        <x:v>Navlungo_Iptal_Tarihi</x:v>
+      </x:c>
+      <x:c r="Y1" t="str">
+        <x:v>Navlungo_Iptal_Sonucu</x:v>
+      </x:c>
+      <x:c r="Z1" t="str">
         <x:v>Kontrol_Uyarısı</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
complete navlungo domestic api integration
</commit_message>
<xml_diff>
--- a/02_SHEET_SISTEM/Tesbih_Kuyusu_V6_5_Ultra_Operasyon_Sheet.xlsx
+++ b/02_SHEET_SISTEM/Tesbih_Kuyusu_V6_5_Ultra_Operasyon_Sheet.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_WHATSAPP_KUYRUGU" sheetId="1" r:id="R39f775ec0a2f497d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ACIK_SIPARISLER" sheetId="2" r:id="R0f2fa0e3c58b4e7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_URUN_KALEMLERI" sheetId="3" r:id="R696493272b8f4bf8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ODEMELER" sheetId="4" r:id="R08bab6b2d1d048ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_FATURA_GRUPLARI" sheetId="5" r:id="Rec6d4b1cff764182"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_PARASUT_FATURA" sheetId="6" r:id="Rda4270abc2d048a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_KARGO_PAKETLERI" sheetId="7" r:id="R123c4f64f662452b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_MUSTERI_HAFIZA" sheetId="8" r:id="Rf1a08fcb98fc45e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_808_FINANS_ONIZLEME" sheetId="9" r:id="Re8df2ba959a0447d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_EBELGE_ISTISNA" sheetId="10" r:id="R23eed220fc4243b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_KONTROL_MERKEZI" sheetId="11" r:id="Rb646dc7e20244b37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_BANKA_HAREKETLERI" sheetId="12" r:id="R5218de48827d45e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_MUSTERI_ADRESLERI" sheetId="13" r:id="R88f30dd4f2634645"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_KULLANIM_KILAVUZU" sheetId="14" r:id="R6e55b4eaf89c45f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_AYARLAR" sheetId="15" r:id="R2c7a89f051f54844"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_VERI_SOZLUGU" sheetId="16" r:id="R4369309b5b0a4ee3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_WHATSAPP_KUYRUGU" sheetId="1" r:id="R29176c4f133e44f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ACIK_SIPARISLER" sheetId="2" r:id="Rebc28217d49f4356"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_URUN_KALEMLERI" sheetId="3" r:id="Re205233853684fe7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ODEMELER" sheetId="4" r:id="R6c70a1d0f5104a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_FATURA_GRUPLARI" sheetId="5" r:id="Raff87fc0044041f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_PARASUT_FATURA" sheetId="6" r:id="R1e898b85c7c54496"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_KARGO_PAKETLERI" sheetId="7" r:id="R2beb48ed65444628"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_MUSTERI_HAFIZA" sheetId="8" r:id="Rf4a82754f6b84582"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_808_FINANS_ONIZLEME" sheetId="9" r:id="R35b120c780924ca2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_EBELGE_ISTISNA" sheetId="10" r:id="R9a056e181e0441c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_KONTROL_MERKEZI" sheetId="11" r:id="Re6fef80ec4a64a23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_BANKA_HAREKETLERI" sheetId="12" r:id="R2ba8cbb7154945fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_MUSTERI_ADRESLERI" sheetId="13" r:id="R369895bd379e4fed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_KULLANIM_KILAVUZU" sheetId="14" r:id="Rc0856524bbe04941"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_AYARLAR" sheetId="15" r:id="Rb8d9f5a8cd8744c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_VERI_SOZLUGU" sheetId="16" r:id="R349b5d4496f04817"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4043,45 +4043,45 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>NAVLUNGO_TEST_MODE</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>Evet</x:v>
-      </x:c>
+        <x:v>NAVLUNGO_SENDER_ADDRESS_ID</x:v>
+      </x:c>
+      <x:c r="B10" t="str"/>
       <x:c r="C10" t="str">
-        <x:v>İlk Navlungo testlerinde kontrollü alıcı kullanılır</x:v>
+        <x:v>Navlungo kayıtlı gönderici adres ID</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="E10" t="str"/>
-      <x:c r="F10" t="str"/>
+      <x:c r="F10" t="str">
+        <x:v>Script Properties önceliklidir</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>NAVLUNGO_SENDER_ADDRESS_ID</x:v>
-      </x:c>
-      <x:c r="B11" t="str"/>
+        <x:v>NAVLUNGO_DEFAULT_CARRIER_ID</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="C11" t="str">
-        <x:v>Navlungo kayıtlı gönderici adres ID</x:v>
+        <x:v>Varsayılan Navlungo taşıyıcı ID</x:v>
       </x:c>
       <x:c r="D11" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="E11" t="str"/>
-      <x:c r="F11" t="str">
-        <x:v>Script Properties önceliklidir</x:v>
-      </x:c>
+      <x:c r="F11" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>NAVLUNGO_DEFAULT_CARRIER_ID</x:v>
+        <x:v>NAVLUNGO_DEFAULT_POST_TYPE</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>Varsayılan Navlungo taşıyıcı ID</x:v>
+        <x:v>Varsayılan Navlungo gönderi tipi</x:v>
       </x:c>
       <x:c r="D12" t="str">
         <x:v>Evet</x:v>
@@ -4091,13 +4091,13 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>NAVLUNGO_DEFAULT_POST_TYPE</x:v>
+        <x:v>NAVLUNGO_DEFAULT_DESI</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>Varsayılan Navlungo gönderi tipi</x:v>
+        <x:v>Varsayılan Navlungo desi</x:v>
       </x:c>
       <x:c r="D13" t="str">
         <x:v>Evet</x:v>
@@ -4107,13 +4107,13 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>NAVLUNGO_DEFAULT_BARCODE_FORMAT</x:v>
+        <x:v>NAVLUNGO_DEFAULT_PACKAGE_COUNT</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>pdf</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>Varsayılan Navlungo barkod formatı</x:v>
+        <x:v>Varsayılan Navlungo paket adedi</x:v>
       </x:c>
       <x:c r="D14" t="str">
         <x:v>Evet</x:v>
@@ -4123,29 +4123,29 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>SISTEM_OPERASYON_SAATI_KAPANIS</x:v>
+        <x:v>NAVLUNGO_CARRIER_ID_MAP_JSON</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>16:00</x:v>
+        <x:v>{}</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>Operasyon kapanış saati</x:v>
+        <x:v>Kargo firması -&gt; Navlungo carrier_id map JSON</x:v>
       </x:c>
       <x:c r="D15" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="E15" t="str"/>
       <x:c r="F15" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>TCKN_VARSAYILAN_GERCEK_KISI</x:v>
+        <x:v>SISTEM_OPERASYON_SAATI_KAPANIS</x:v>
       </x:c>
       <x:c r="B16" t="str">
-        <x:v>11111111111</x:v>
+        <x:v>16:00</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>Gerçek kişi TCKN boşsa uygulanabilir</x:v>
+        <x:v>Operasyon kapanış saati</x:v>
       </x:c>
       <x:c r="D16" t="str">
         <x:v>Evet</x:v>
@@ -4155,13 +4155,13 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>BANKA_HAREKET_MODULU_AKTIF</x:v>
+        <x:v>TCKN_VARSAYILAN_GERCEK_KISI</x:v>
       </x:c>
       <x:c r="B17" t="str">
-        <x:v>Evet</x:v>
+        <x:v>11111111111</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>14 banka hareketi teyit katmanı</x:v>
+        <x:v>Gerçek kişi TCKN boşsa uygulanabilir</x:v>
       </x:c>
       <x:c r="D17" t="str">
         <x:v>Evet</x:v>
@@ -4171,35 +4171,51 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>VARSAYILAN_KARGO_FIRMASI</x:v>
+        <x:v>BANKA_HAREKET_MODULU_AKTIF</x:v>
       </x:c>
       <x:c r="B18" t="str">
-        <x:v>Aras Kargo</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="C18" t="str">
-        <x:v>Kargo firması önerisi</x:v>
+        <x:v>14 banka hareketi teyit katmanı</x:v>
       </x:c>
       <x:c r="D18" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="E18" t="str"/>
       <x:c r="F18" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>KARGO_UCRETI_STANDART</x:v>
+        <x:v>VARSAYILAN_KARGO_FIRMASI</x:v>
       </x:c>
       <x:c r="B19" t="str">
-        <x:v>125</x:v>
+        <x:v>Aras Kargo</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>808 finans ön izleme için varsayılan maliyet</x:v>
+        <x:v>Kargo firması önerisi</x:v>
       </x:c>
       <x:c r="D19" t="str">
         <x:v>Hayır</x:v>
       </x:c>
       <x:c r="E19" t="str"/>
       <x:c r="F19" t="str"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>KARGO_UCRETI_STANDART</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>808 finans ön izleme için varsayılan maliyet</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="E20" t="str"/>
+      <x:c r="F20" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7355,16 +7371,16 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B158" t="str">
-        <x:v>Navlungo_Gonderi_ID</x:v>
+        <x:v>Navlungo_Post_Number</x:v>
       </x:c>
       <x:c r="C158" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D158" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E158" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F158" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7375,16 +7391,16 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B159" t="str">
-        <x:v>Navlungo_Barkod_No</x:v>
+        <x:v>Navlungo_Reference_ID</x:v>
       </x:c>
       <x:c r="C159" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D159" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E159" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F159" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7395,7 +7411,7 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B160" t="str">
-        <x:v>Navlungo_Takip_No</x:v>
+        <x:v>Navlungo_Tracking_URL</x:v>
       </x:c>
       <x:c r="C160" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
@@ -7415,7 +7431,7 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B161" t="str">
-        <x:v>Navlungo_Etiket_URL</x:v>
+        <x:v>Navlungo_Barcode_URL</x:v>
       </x:c>
       <x:c r="C161" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
@@ -7435,13 +7451,13 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B162" t="str">
-        <x:v>Navlungo_Durum</x:v>
+        <x:v>Navlungo_Carrier_ID</x:v>
       </x:c>
       <x:c r="C162" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D162" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E162" t="str">
         <x:v>Evet</x:v>
@@ -7455,13 +7471,13 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B163" t="str">
-        <x:v>Navlungo_Hata_Mesaji</x:v>
+        <x:v>Navlungo_Carrier_Name</x:v>
       </x:c>
       <x:c r="C163" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D163" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E163" t="str">
         <x:v>Hayır</x:v>
@@ -7475,7 +7491,7 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B164" t="str">
-        <x:v>Navlungo_Payload_JSON</x:v>
+        <x:v>Navlungo_Status</x:v>
       </x:c>
       <x:c r="C164" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
@@ -7495,7 +7511,7 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B165" t="str">
-        <x:v>Navlungo_Response_JSON</x:v>
+        <x:v>Navlungo_Last_Response</x:v>
       </x:c>
       <x:c r="C165" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
@@ -7515,13 +7531,13 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B166" t="str">
-        <x:v>Test_Kargo_Mu</x:v>
+        <x:v>Navlungo_Last_Error</x:v>
       </x:c>
       <x:c r="C166" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D166" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E166" t="str">
         <x:v>Hayır</x:v>
@@ -7535,13 +7551,13 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B167" t="str">
-        <x:v>Navlungo_Olusturma_Tarihi</x:v>
+        <x:v>Navlungo_Created_At</x:v>
       </x:c>
       <x:c r="C167" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D167" t="str">
-        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E167" t="str">
         <x:v>Hayır</x:v>
@@ -7555,13 +7571,13 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B168" t="str">
-        <x:v>Navlungo_Iptal_Tarihi</x:v>
+        <x:v>Navlungo_Cancelled_At</x:v>
       </x:c>
       <x:c r="C168" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D168" t="str">
-        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E168" t="str">
         <x:v>Hayır</x:v>
@@ -7575,7 +7591,7 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B169" t="str">
-        <x:v>Navlungo_Iptal_Sonucu</x:v>
+        <x:v>Navlungo_Test_Mu</x:v>
       </x:c>
       <x:c r="C169" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
@@ -7595,13 +7611,13 @@
         <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B170" t="str">
-        <x:v>Kontrol_Uyarısı</x:v>
+        <x:v>Navlungo_Payload_Hash</x:v>
       </x:c>
       <x:c r="C170" t="str">
         <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D170" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E170" t="str">
         <x:v>Hayır</x:v>
@@ -7612,19 +7628,19 @@
     </x:row>
     <x:row r="171">
       <x:c r="A171" t="str">
-        <x:v>09_MUSTERI_HAFIZA</x:v>
+        <x:v>08_KARGO_PAKETLERI</x:v>
       </x:c>
       <x:c r="B171" t="str">
-        <x:v>WhatsApp_Tel</x:v>
+        <x:v>Kontrol_Uyarısı</x:v>
       </x:c>
       <x:c r="C171" t="str">
-        <x:v>Müşteri hafıza motoru</x:v>
+        <x:v>Ultra panel / Kargo bilgisi gir / kargo motoru</x:v>
       </x:c>
       <x:c r="D171" t="str">
-        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E171" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F171" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7635,16 +7651,16 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B172" t="str">
-        <x:v>Sipariş_Sahibi</x:v>
+        <x:v>WhatsApp_Tel</x:v>
       </x:c>
       <x:c r="C172" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D172" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
       </x:c>
       <x:c r="E172" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F172" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7655,13 +7671,13 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B173" t="str">
-        <x:v>Son_Kargo_Alıcısı</x:v>
+        <x:v>Sipariş_Sahibi</x:v>
       </x:c>
       <x:c r="C173" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D173" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E173" t="str">
         <x:v>Hayır</x:v>
@@ -7675,16 +7691,16 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B174" t="str">
-        <x:v>Son_Kargo_Tel</x:v>
+        <x:v>Son_Kargo_Alıcısı</x:v>
       </x:c>
       <x:c r="C174" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D174" t="str">
-        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E174" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F174" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7695,16 +7711,16 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B175" t="str">
-        <x:v>Son_İl</x:v>
+        <x:v>Son_Kargo_Tel</x:v>
       </x:c>
       <x:c r="C175" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D175" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
       </x:c>
       <x:c r="E175" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F175" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7715,7 +7731,7 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B176" t="str">
-        <x:v>Son_İlçe</x:v>
+        <x:v>Son_İl</x:v>
       </x:c>
       <x:c r="C176" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
@@ -7735,7 +7751,7 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B177" t="str">
-        <x:v>Son_Adres</x:v>
+        <x:v>Son_İlçe</x:v>
       </x:c>
       <x:c r="C177" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
@@ -7755,13 +7771,13 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B178" t="str">
-        <x:v>Son_Fatura_Kişisi</x:v>
+        <x:v>Son_Adres</x:v>
       </x:c>
       <x:c r="C178" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D178" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E178" t="str">
         <x:v>Hayır</x:v>
@@ -7775,16 +7791,16 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B179" t="str">
-        <x:v>Son_Fatura_Tel</x:v>
+        <x:v>Son_Fatura_Kişisi</x:v>
       </x:c>
       <x:c r="C179" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D179" t="str">
-        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E179" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F179" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7795,16 +7811,16 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B180" t="str">
-        <x:v>Son_Fatura_TCKN_VKN</x:v>
+        <x:v>Son_Fatura_Tel</x:v>
       </x:c>
       <x:c r="C180" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D180" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
       </x:c>
       <x:c r="E180" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F180" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7815,16 +7831,16 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B181" t="str">
-        <x:v>Paraşüt_Cari_ID</x:v>
+        <x:v>Son_Fatura_TCKN_VKN</x:v>
       </x:c>
       <x:c r="C181" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D181" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E181" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F181" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7835,16 +7851,16 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B182" t="str">
-        <x:v>Son_Ödeme_Yapanlar_JSON</x:v>
+        <x:v>Paraşüt_Cari_ID</x:v>
       </x:c>
       <x:c r="C182" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D182" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E182" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F182" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7855,13 +7871,13 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B183" t="str">
-        <x:v>Cari_Adaylari_JSON</x:v>
+        <x:v>Son_Ödeme_Yapanlar_JSON</x:v>
       </x:c>
       <x:c r="C183" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D183" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E183" t="str">
         <x:v>Hayır</x:v>
@@ -7875,13 +7891,13 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B184" t="str">
-        <x:v>Son_Kargo_Bilgisi_JSON</x:v>
+        <x:v>Cari_Adaylari_JSON</x:v>
       </x:c>
       <x:c r="C184" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D184" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E184" t="str">
         <x:v>Hayır</x:v>
@@ -7895,13 +7911,13 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B185" t="str">
-        <x:v>Güven_Puanı</x:v>
+        <x:v>Son_Kargo_Bilgisi_JSON</x:v>
       </x:c>
       <x:c r="C185" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D185" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E185" t="str">
         <x:v>Hayır</x:v>
@@ -7915,16 +7931,16 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B186" t="str">
-        <x:v>Son_Başarılı_Sipariş_ID</x:v>
+        <x:v>Güven_Puanı</x:v>
       </x:c>
       <x:c r="C186" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D186" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E186" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F186" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7935,16 +7951,16 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B187" t="str">
-        <x:v>Son_Güncelleme</x:v>
+        <x:v>Son_Başarılı_Sipariş_ID</x:v>
       </x:c>
       <x:c r="C187" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D187" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E187" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F187" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -7955,13 +7971,13 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B188" t="str">
-        <x:v>Güven_Notu</x:v>
+        <x:v>Son_Güncelleme</x:v>
       </x:c>
       <x:c r="C188" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D188" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E188" t="str">
         <x:v>Hayır</x:v>
@@ -7975,7 +7991,7 @@
         <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B189" t="str">
-        <x:v>Kontrol_Uyarısı</x:v>
+        <x:v>Güven_Notu</x:v>
       </x:c>
       <x:c r="C189" t="str">
         <x:v>Müşteri hafıza motoru</x:v>
@@ -7992,19 +8008,19 @@
     </x:row>
     <x:row r="190">
       <x:c r="A190" t="str">
-        <x:v>10_808_FINANS_ONIZLEME</x:v>
+        <x:v>09_MUSTERI_HAFIZA</x:v>
       </x:c>
       <x:c r="B190" t="str">
-        <x:v>808_Kayıt_ID</x:v>
+        <x:v>Kontrol_Uyarısı</x:v>
       </x:c>
       <x:c r="C190" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Müşteri hafıza motoru</x:v>
       </x:c>
       <x:c r="D190" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E190" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F190" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8015,7 +8031,7 @@
         <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B191" t="str">
-        <x:v>Açık_Sipariş_ID</x:v>
+        <x:v>808_Kayıt_ID</x:v>
       </x:c>
       <x:c r="C191" t="str">
         <x:v>Sistem</x:v>
@@ -8035,16 +8051,16 @@
         <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B192" t="str">
-        <x:v>Model_Tipi</x:v>
+        <x:v>Açık_Sipariş_ID</x:v>
       </x:c>
       <x:c r="C192" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D192" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E192" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F192" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8055,13 +8071,13 @@
         <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B193" t="str">
-        <x:v>Ürün_Toplamı</x:v>
+        <x:v>Model_Tipi</x:v>
       </x:c>
       <x:c r="C193" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D193" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E193" t="str">
         <x:v>Hayır</x:v>
@@ -8075,7 +8091,7 @@
         <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B194" t="str">
-        <x:v>KDV_Hariç</x:v>
+        <x:v>Ürün_Toplamı</x:v>
       </x:c>
       <x:c r="C194" t="str">
         <x:v>Sistem</x:v>
@@ -8095,7 +8111,7 @@
         <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B195" t="str">
-        <x:v>KDV_Tutarı</x:v>
+        <x:v>KDV_Hariç</x:v>
       </x:c>
       <x:c r="C195" t="str">
         <x:v>Sistem</x:v>
@@ -8104,7 +8120,7 @@
         <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E195" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F195" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8115,7 +8131,7 @@
         <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B196" t="str">
-        <x:v>Ödeme_Toplamı</x:v>
+        <x:v>KDV_Tutarı</x:v>
       </x:c>
       <x:c r="C196" t="str">
         <x:v>Sistem</x:v>
@@ -8124,7 +8140,7 @@
         <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E196" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F196" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8135,7 +8151,7 @@
         <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B197" t="str">
-        <x:v>Fark</x:v>
+        <x:v>Ödeme_Toplamı</x:v>
       </x:c>
       <x:c r="C197" t="str">
         <x:v>Sistem</x:v>
@@ -8155,13 +8171,13 @@
         <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B198" t="str">
-        <x:v>Net_Ticari_Kazanç</x:v>
+        <x:v>Fark</x:v>
       </x:c>
       <x:c r="C198" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D198" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E198" t="str">
         <x:v>Hayır</x:v>
@@ -8175,13 +8191,13 @@
         <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B199" t="str">
-        <x:v>Resmi_Fatura_Notu</x:v>
+        <x:v>Net_Ticari_Kazanç</x:v>
       </x:c>
       <x:c r="C199" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D199" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E199" t="str">
         <x:v>Hayır</x:v>
@@ -8195,7 +8211,7 @@
         <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B200" t="str">
-        <x:v>Fatura_Etkisi_Yok</x:v>
+        <x:v>Resmi_Fatura_Notu</x:v>
       </x:c>
       <x:c r="C200" t="str">
         <x:v>Sistem</x:v>
@@ -8215,13 +8231,13 @@
         <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B201" t="str">
-        <x:v>Kontrol_Uyarısı</x:v>
+        <x:v>Fatura_Etkisi_Yok</x:v>
       </x:c>
       <x:c r="C201" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D201" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E201" t="str">
         <x:v>Hayır</x:v>
@@ -8232,19 +8248,19 @@
     </x:row>
     <x:row r="202">
       <x:c r="A202" t="str">
-        <x:v>11_EBELGE_ISTISNA</x:v>
+        <x:v>10_808_FINANS_ONIZLEME</x:v>
       </x:c>
       <x:c r="B202" t="str">
-        <x:v>E_Belge_Kayıt_ID</x:v>
+        <x:v>Kontrol_Uyarısı</x:v>
       </x:c>
       <x:c r="C202" t="str">
-        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
+        <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D202" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E202" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F202" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8255,7 +8271,7 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B203" t="str">
-        <x:v>Fatura_Grubu_ID</x:v>
+        <x:v>E_Belge_Kayıt_ID</x:v>
       </x:c>
       <x:c r="C203" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
@@ -8275,7 +8291,7 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B204" t="str">
-        <x:v>Açık_Sipariş_ID</x:v>
+        <x:v>Fatura_Grubu_ID</x:v>
       </x:c>
       <x:c r="C204" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
@@ -8295,7 +8311,7 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B205" t="str">
-        <x:v>Paraşüt_Fatura_ID</x:v>
+        <x:v>Açık_Sipariş_ID</x:v>
       </x:c>
       <x:c r="C205" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
@@ -8315,16 +8331,16 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B206" t="str">
-        <x:v>Fatura_Kişisi</x:v>
+        <x:v>Paraşüt_Fatura_ID</x:v>
       </x:c>
       <x:c r="C206" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D206" t="str">
-        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E206" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F206" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8335,7 +8351,7 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B207" t="str">
-        <x:v>Fatura_TCKN_VKN</x:v>
+        <x:v>Fatura_Kişisi</x:v>
       </x:c>
       <x:c r="C207" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
@@ -8355,7 +8371,7 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B208" t="str">
-        <x:v>Cari_Tipi</x:v>
+        <x:v>Fatura_TCKN_VKN</x:v>
       </x:c>
       <x:c r="C208" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
@@ -8375,13 +8391,13 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B209" t="str">
-        <x:v>E_Belge_Tipi</x:v>
+        <x:v>Cari_Tipi</x:v>
       </x:c>
       <x:c r="C209" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D209" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Fatura, cari ve Paraşüt taslak hazırlığını desteklemek</x:v>
       </x:c>
       <x:c r="E209" t="str">
         <x:v>Hayır</x:v>
@@ -8395,7 +8411,7 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B210" t="str">
-        <x:v>Gümüş_İçeriyor_Mu</x:v>
+        <x:v>E_Belge_Tipi</x:v>
       </x:c>
       <x:c r="C210" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
@@ -8415,13 +8431,13 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B211" t="str">
-        <x:v>KDV0_Satırı_Var_Mı</x:v>
+        <x:v>Gümüş_İçeriyor_Mu</x:v>
       </x:c>
       <x:c r="C211" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D211" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E211" t="str">
         <x:v>Hayır</x:v>
@@ -8435,13 +8451,13 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B212" t="str">
-        <x:v>İstisna_Gerekli_Mi</x:v>
+        <x:v>KDV0_Satırı_Var_Mı</x:v>
       </x:c>
       <x:c r="C212" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D212" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E212" t="str">
         <x:v>Hayır</x:v>
@@ -8455,7 +8471,7 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B213" t="str">
-        <x:v>İstisna_Kodu</x:v>
+        <x:v>İstisna_Gerekli_Mi</x:v>
       </x:c>
       <x:c r="C213" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
@@ -8464,7 +8480,7 @@
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E213" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F213" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8475,16 +8491,16 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B214" t="str">
-        <x:v>İstisna_Açıklama</x:v>
+        <x:v>İstisna_Kodu</x:v>
       </x:c>
       <x:c r="C214" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D214" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E214" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F214" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8495,16 +8511,16 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B215" t="str">
-        <x:v>Gönderim_Durumu</x:v>
+        <x:v>İstisna_Açıklama</x:v>
       </x:c>
       <x:c r="C215" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D215" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E215" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F215" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8515,7 +8531,7 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B216" t="str">
-        <x:v>Resmi_Gönderim_Onayı</x:v>
+        <x:v>Gönderim_Durumu</x:v>
       </x:c>
       <x:c r="C216" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
@@ -8524,7 +8540,7 @@
         <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E216" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F216" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8535,7 +8551,7 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B217" t="str">
-        <x:v>Resmi_Gönderim_Blokaj_Nedeni</x:v>
+        <x:v>Resmi_Gönderim_Onayı</x:v>
       </x:c>
       <x:c r="C217" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
@@ -8555,13 +8571,13 @@
         <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B218" t="str">
-        <x:v>Kontrol_Seviyesi</x:v>
+        <x:v>Resmi_Gönderim_Blokaj_Nedeni</x:v>
       </x:c>
       <x:c r="C218" t="str">
         <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D218" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E218" t="str">
         <x:v>Hayır</x:v>
@@ -8572,19 +8588,19 @@
     </x:row>
     <x:row r="219">
       <x:c r="A219" t="str">
-        <x:v>12_KONTROL_MERKEZI</x:v>
+        <x:v>11_EBELGE_ISTISNA</x:v>
       </x:c>
       <x:c r="B219" t="str">
-        <x:v>Kontrol_ID</x:v>
+        <x:v>Kontrol_Seviyesi</x:v>
       </x:c>
       <x:c r="C219" t="str">
-        <x:v>Kontrol merkezi motoru</x:v>
+        <x:v>e-Belge ve istisna hazırlık motoru</x:v>
       </x:c>
       <x:c r="D219" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E219" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F219" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8595,16 +8611,16 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B220" t="str">
-        <x:v>Tarih</x:v>
+        <x:v>Kontrol_ID</x:v>
       </x:c>
       <x:c r="C220" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D220" t="str">
-        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E220" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F220" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8615,13 +8631,13 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B221" t="str">
-        <x:v>Kaynak_Sayfa</x:v>
+        <x:v>Tarih</x:v>
       </x:c>
       <x:c r="C221" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D221" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
       </x:c>
       <x:c r="E221" t="str">
         <x:v>Hayır</x:v>
@@ -8635,16 +8651,16 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B222" t="str">
-        <x:v>Kaynak_ID</x:v>
+        <x:v>Kaynak_Sayfa</x:v>
       </x:c>
       <x:c r="C222" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D222" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E222" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F222" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8655,16 +8671,16 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B223" t="str">
-        <x:v>Kontrol_Tipi</x:v>
+        <x:v>Kaynak_ID</x:v>
       </x:c>
       <x:c r="C223" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D223" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E223" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F223" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8675,7 +8691,7 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B224" t="str">
-        <x:v>Risk_Seviyesi</x:v>
+        <x:v>Kontrol_Tipi</x:v>
       </x:c>
       <x:c r="C224" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
@@ -8695,16 +8711,16 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B225" t="str">
-        <x:v>Durum</x:v>
+        <x:v>Risk_Seviyesi</x:v>
       </x:c>
       <x:c r="C225" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D225" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E225" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F225" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8715,16 +8731,16 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B226" t="str">
-        <x:v>Kontrol_Uyarısı</x:v>
+        <x:v>Durum</x:v>
       </x:c>
       <x:c r="C226" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D226" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E226" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F226" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8735,7 +8751,7 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B227" t="str">
-        <x:v>Beklenen_Aksiyon</x:v>
+        <x:v>Kontrol_Uyarısı</x:v>
       </x:c>
       <x:c r="C227" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
@@ -8755,13 +8771,13 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B228" t="str">
-        <x:v>Sorumlu</x:v>
+        <x:v>Beklenen_Aksiyon</x:v>
       </x:c>
       <x:c r="C228" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D228" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E228" t="str">
         <x:v>Hayır</x:v>
@@ -8775,13 +8791,13 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B229" t="str">
-        <x:v>Çözüm_Notu</x:v>
+        <x:v>Sorumlu</x:v>
       </x:c>
       <x:c r="C229" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D229" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E229" t="str">
         <x:v>Hayır</x:v>
@@ -8795,13 +8811,13 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B230" t="str">
-        <x:v>Kapanış_Tarihi</x:v>
+        <x:v>Çözüm_Notu</x:v>
       </x:c>
       <x:c r="C230" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D230" t="str">
-        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E230" t="str">
         <x:v>Hayır</x:v>
@@ -8815,13 +8831,13 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B231" t="str">
-        <x:v>Blokaj_Mı</x:v>
+        <x:v>Kapanış_Tarihi</x:v>
       </x:c>
       <x:c r="C231" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D231" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
       </x:c>
       <x:c r="E231" t="str">
         <x:v>Hayır</x:v>
@@ -8835,13 +8851,13 @@
         <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B232" t="str">
-        <x:v>İlgili_Modül</x:v>
+        <x:v>Blokaj_Mı</x:v>
       </x:c>
       <x:c r="C232" t="str">
         <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D232" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E232" t="str">
         <x:v>Hayır</x:v>
@@ -8852,16 +8868,16 @@
     </x:row>
     <x:row r="233">
       <x:c r="A233" t="str">
-        <x:v>13_VERI_SOZLUGU</x:v>
+        <x:v>12_KONTROL_MERKEZI</x:v>
       </x:c>
       <x:c r="B233" t="str">
-        <x:v>Sayfa</x:v>
+        <x:v>İlgili_Modül</x:v>
       </x:c>
       <x:c r="C233" t="str">
-        <x:v>Koddan üretilen kolon sözlüğü</x:v>
+        <x:v>Kontrol merkezi motoru</x:v>
       </x:c>
       <x:c r="D233" t="str">
-        <x:v>Veri sözlüğü alanını tanımlamak</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E233" t="str">
         <x:v>Hayır</x:v>
@@ -8875,7 +8891,7 @@
         <x:v>13_VERI_SOZLUGU</x:v>
       </x:c>
       <x:c r="B234" t="str">
-        <x:v>Kolon</x:v>
+        <x:v>Sayfa</x:v>
       </x:c>
       <x:c r="C234" t="str">
         <x:v>Koddan üretilen kolon sözlüğü</x:v>
@@ -8895,7 +8911,7 @@
         <x:v>13_VERI_SOZLUGU</x:v>
       </x:c>
       <x:c r="B235" t="str">
-        <x:v>Kaynak</x:v>
+        <x:v>Kolon</x:v>
       </x:c>
       <x:c r="C235" t="str">
         <x:v>Koddan üretilen kolon sözlüğü</x:v>
@@ -8915,7 +8931,7 @@
         <x:v>13_VERI_SOZLUGU</x:v>
       </x:c>
       <x:c r="B236" t="str">
-        <x:v>Amaç</x:v>
+        <x:v>Kaynak</x:v>
       </x:c>
       <x:c r="C236" t="str">
         <x:v>Koddan üretilen kolon sözlüğü</x:v>
@@ -8935,7 +8951,7 @@
         <x:v>13_VERI_SOZLUGU</x:v>
       </x:c>
       <x:c r="B237" t="str">
-        <x:v>Zorunlu_Mu</x:v>
+        <x:v>Amaç</x:v>
       </x:c>
       <x:c r="C237" t="str">
         <x:v>Koddan üretilen kolon sözlüğü</x:v>
@@ -8955,13 +8971,13 @@
         <x:v>13_VERI_SOZLUGU</x:v>
       </x:c>
       <x:c r="B238" t="str">
-        <x:v>Not</x:v>
+        <x:v>Zorunlu_Mu</x:v>
       </x:c>
       <x:c r="C238" t="str">
         <x:v>Koddan üretilen kolon sözlüğü</x:v>
       </x:c>
       <x:c r="D238" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>Veri sözlüğü alanını tanımlamak</x:v>
       </x:c>
       <x:c r="E238" t="str">
         <x:v>Hayır</x:v>
@@ -8972,19 +8988,19 @@
     </x:row>
     <x:row r="239">
       <x:c r="A239" t="str">
-        <x:v>14_BANKA_HAREKETLERI</x:v>
+        <x:v>13_VERI_SOZLUGU</x:v>
       </x:c>
       <x:c r="B239" t="str">
-        <x:v>Banka_Hareket_ID</x:v>
+        <x:v>Not</x:v>
       </x:c>
       <x:c r="C239" t="str">
-        <x:v>Manuel banka hareketi içeri alma</x:v>
+        <x:v>Koddan üretilen kolon sözlüğü</x:v>
       </x:c>
       <x:c r="D239" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E239" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F239" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -8995,16 +9011,16 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B240" t="str">
-        <x:v>İşlem_Tarihi</x:v>
+        <x:v>Banka_Hareket_ID</x:v>
       </x:c>
       <x:c r="C240" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D240" t="str">
-        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E240" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F240" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9015,7 +9031,7 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B241" t="str">
-        <x:v>Valör_Tarihi</x:v>
+        <x:v>İşlem_Tarihi</x:v>
       </x:c>
       <x:c r="C241" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
@@ -9035,16 +9051,16 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B242" t="str">
-        <x:v>Gönderen_Adı</x:v>
+        <x:v>Valör_Tarihi</x:v>
       </x:c>
       <x:c r="C242" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D242" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Operasyon tarih ve zaman bilgisini tutmak</x:v>
       </x:c>
       <x:c r="E242" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F242" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9055,16 +9071,16 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B243" t="str">
-        <x:v>Açıklama</x:v>
+        <x:v>Gönderen_Adı</x:v>
       </x:c>
       <x:c r="C243" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D243" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E243" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F243" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9075,16 +9091,16 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B244" t="str">
-        <x:v>Tutar</x:v>
+        <x:v>Açıklama</x:v>
       </x:c>
       <x:c r="C244" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D244" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E244" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F244" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9095,13 +9111,13 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B245" t="str">
-        <x:v>Banka_Adı</x:v>
+        <x:v>Tutar</x:v>
       </x:c>
       <x:c r="C245" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D245" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E245" t="str">
         <x:v>Evet</x:v>
@@ -9115,7 +9131,7 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B246" t="str">
-        <x:v>IBAN</x:v>
+        <x:v>Banka_Adı</x:v>
       </x:c>
       <x:c r="C246" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
@@ -9124,7 +9140,7 @@
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E246" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F246" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9135,7 +9151,7 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B247" t="str">
-        <x:v>İşlem_Tipi</x:v>
+        <x:v>IBAN</x:v>
       </x:c>
       <x:c r="C247" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
@@ -9155,7 +9171,7 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B248" t="str">
-        <x:v>Referans_No</x:v>
+        <x:v>İşlem_Tipi</x:v>
       </x:c>
       <x:c r="C248" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
@@ -9175,16 +9191,16 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B249" t="str">
-        <x:v>Eşleşme_Durumu</x:v>
+        <x:v>Referans_No</x:v>
       </x:c>
       <x:c r="C249" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D249" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E249" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F249" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9195,16 +9211,16 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B250" t="str">
-        <x:v>Eşleşme_Puanı</x:v>
+        <x:v>Eşleşme_Durumu</x:v>
       </x:c>
       <x:c r="C250" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D250" t="str">
-        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E250" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F250" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9215,16 +9231,16 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B251" t="str">
-        <x:v>Önerilen_Açık_Sipariş_ID</x:v>
+        <x:v>Eşleşme_Puanı</x:v>
       </x:c>
       <x:c r="C251" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D251" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Finansal, miktarsal veya kontrol hesaplamasını taşımak</x:v>
       </x:c>
       <x:c r="E251" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F251" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9235,7 +9251,7 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B252" t="str">
-        <x:v>Önerilen_Ödeme_ID</x:v>
+        <x:v>Önerilen_Açık_Sipariş_ID</x:v>
       </x:c>
       <x:c r="C252" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
@@ -9255,16 +9271,16 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B253" t="str">
-        <x:v>Önerilen_Ödeme_Yapan</x:v>
+        <x:v>Önerilen_Ödeme_ID</x:v>
       </x:c>
       <x:c r="C253" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D253" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E253" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F253" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9275,13 +9291,13 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B254" t="str">
-        <x:v>Operatör_Onayı</x:v>
+        <x:v>Önerilen_Ödeme_Yapan</x:v>
       </x:c>
       <x:c r="C254" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D254" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E254" t="str">
         <x:v>Hayır</x:v>
@@ -9295,13 +9311,13 @@
         <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B255" t="str">
-        <x:v>Kontrol_Uyarısı</x:v>
+        <x:v>Operatör_Onayı</x:v>
       </x:c>
       <x:c r="C255" t="str">
         <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D255" t="str">
-        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
       </x:c>
       <x:c r="E255" t="str">
         <x:v>Hayır</x:v>
@@ -9312,19 +9328,19 @@
     </x:row>
     <x:row r="256">
       <x:c r="A256" t="str">
-        <x:v>15_MUSTERI_ADRESLERI</x:v>
+        <x:v>14_BANKA_HAREKETLERI</x:v>
       </x:c>
       <x:c r="B256" t="str">
-        <x:v>Adres_ID</x:v>
+        <x:v>Kontrol_Uyarısı</x:v>
       </x:c>
       <x:c r="C256" t="str">
-        <x:v>Sistem</x:v>
+        <x:v>Manuel banka hareketi içeri alma</x:v>
       </x:c>
       <x:c r="D256" t="str">
-        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
+        <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
       <x:c r="E256" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F256" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9335,13 +9351,13 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B257" t="str">
-        <x:v>WhatsApp_Tel</x:v>
+        <x:v>Adres_ID</x:v>
       </x:c>
       <x:c r="C257" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D257" t="str">
-        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
+        <x:v>Kayıtları benzersiz bağlamak ve ilişkileri kurmak</x:v>
       </x:c>
       <x:c r="E257" t="str">
         <x:v>Evet</x:v>
@@ -9355,16 +9371,16 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B258" t="str">
-        <x:v>Sipariş_Sahibi</x:v>
+        <x:v>WhatsApp_Tel</x:v>
       </x:c>
       <x:c r="C258" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D258" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
       </x:c>
       <x:c r="E258" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F258" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9375,13 +9391,13 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B259" t="str">
-        <x:v>Kargo_Alıcısı</x:v>
+        <x:v>Sipariş_Sahibi</x:v>
       </x:c>
       <x:c r="C259" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D259" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E259" t="str">
         <x:v>Hayır</x:v>
@@ -9395,16 +9411,16 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B260" t="str">
-        <x:v>Kargo_Tel</x:v>
+        <x:v>Kargo_Alıcısı</x:v>
       </x:c>
       <x:c r="C260" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D260" t="str">
-        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E260" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F260" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9415,16 +9431,16 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B261" t="str">
-        <x:v>İl</x:v>
+        <x:v>Kargo_Tel</x:v>
       </x:c>
       <x:c r="C261" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D261" t="str">
-        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
+        <x:v>Telefon bilgisini normalize ederek eşleşme ve iletişimde kullanmak</x:v>
       </x:c>
       <x:c r="E261" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="F261" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9435,7 +9451,7 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B262" t="str">
-        <x:v>İlçe</x:v>
+        <x:v>İl</x:v>
       </x:c>
       <x:c r="C262" t="str">
         <x:v>Sistem</x:v>
@@ -9455,7 +9471,7 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B263" t="str">
-        <x:v>Adres</x:v>
+        <x:v>İlçe</x:v>
       </x:c>
       <x:c r="C263" t="str">
         <x:v>Sistem</x:v>
@@ -9475,7 +9491,7 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B264" t="str">
-        <x:v>Kargo_Firması</x:v>
+        <x:v>Adres</x:v>
       </x:c>
       <x:c r="C264" t="str">
         <x:v>Sistem</x:v>
@@ -9495,13 +9511,13 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B265" t="str">
-        <x:v>Varsayılan_Mı</x:v>
+        <x:v>Kargo_Firması</x:v>
       </x:c>
       <x:c r="C265" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D265" t="str">
-        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
+        <x:v>Kargo ve adres operasyon bilgisini taşımak</x:v>
       </x:c>
       <x:c r="E265" t="str">
         <x:v>Hayır</x:v>
@@ -9515,7 +9531,7 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B266" t="str">
-        <x:v>Son_Kullanım</x:v>
+        <x:v>Varsayılan_Mı</x:v>
       </x:c>
       <x:c r="C266" t="str">
         <x:v>Sistem</x:v>
@@ -9535,16 +9551,16 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B267" t="str">
-        <x:v>Adres_Durumu</x:v>
+        <x:v>Son_Kullanım</x:v>
       </x:c>
       <x:c r="C267" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D267" t="str">
-        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi kapsamında veri alanını taşımak</x:v>
       </x:c>
       <x:c r="E267" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="F267" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
@@ -9555,18 +9571,38 @@
         <x:v>15_MUSTERI_ADRESLERI</x:v>
       </x:c>
       <x:c r="B268" t="str">
-        <x:v>Kontrol_Uyarısı</x:v>
+        <x:v>Adres_Durumu</x:v>
       </x:c>
       <x:c r="C268" t="str">
         <x:v>Sistem</x:v>
       </x:c>
       <x:c r="D268" t="str">
+        <x:v>Süreç durumunu, kilidi veya operatör onayını göstermek</x:v>
+      </x:c>
+      <x:c r="E268" t="str">
+        <x:v>Evet</x:v>
+      </x:c>
+      <x:c r="F268" t="str">
+        <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269">
+      <x:c r="A269" t="str">
+        <x:v>15_MUSTERI_ADRESLERI</x:v>
+      </x:c>
+      <x:c r="B269" t="str">
+        <x:v>Kontrol_Uyarısı</x:v>
+      </x:c>
+      <x:c r="C269" t="str">
+        <x:v>Sistem</x:v>
+      </x:c>
+      <x:c r="D269" t="str">
         <x:v>Operatöre kontrol, uyarı veya aksiyon bilgisi vermek</x:v>
       </x:c>
-      <x:c r="E268" t="str">
-        <x:v>Hayır</x:v>
-      </x:c>
-      <x:c r="F268" t="str">
+      <x:c r="E269" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="F269" t="str">
         <x:v>V6.5 Ultra Operasyon kolon sözleşmesi</x:v>
       </x:c>
     </x:row>
@@ -15198,42 +15234,45 @@
         <x:v>Paket_Notu</x:v>
       </x:c>
       <x:c r="N1" s="13" t="str">
-        <x:v>Navlungo_Gonderi_ID</x:v>
+        <x:v>Navlungo_Post_Number</x:v>
       </x:c>
       <x:c r="O1" t="str">
-        <x:v>Navlungo_Barkod_No</x:v>
+        <x:v>Navlungo_Reference_ID</x:v>
       </x:c>
       <x:c r="P1" t="str">
-        <x:v>Navlungo_Takip_No</x:v>
+        <x:v>Navlungo_Tracking_URL</x:v>
       </x:c>
       <x:c r="Q1" t="str">
-        <x:v>Navlungo_Etiket_URL</x:v>
+        <x:v>Navlungo_Barcode_URL</x:v>
       </x:c>
       <x:c r="R1" t="str">
-        <x:v>Navlungo_Durum</x:v>
+        <x:v>Navlungo_Carrier_ID</x:v>
       </x:c>
       <x:c r="S1" t="str">
-        <x:v>Navlungo_Hata_Mesaji</x:v>
+        <x:v>Navlungo_Carrier_Name</x:v>
       </x:c>
       <x:c r="T1" t="str">
-        <x:v>Navlungo_Payload_JSON</x:v>
+        <x:v>Navlungo_Status</x:v>
       </x:c>
       <x:c r="U1" t="str">
-        <x:v>Navlungo_Response_JSON</x:v>
+        <x:v>Navlungo_Last_Response</x:v>
       </x:c>
       <x:c r="V1" t="str">
-        <x:v>Test_Kargo_Mu</x:v>
+        <x:v>Navlungo_Last_Error</x:v>
       </x:c>
       <x:c r="W1" t="str">
-        <x:v>Navlungo_Olusturma_Tarihi</x:v>
+        <x:v>Navlungo_Created_At</x:v>
       </x:c>
       <x:c r="X1" t="str">
-        <x:v>Navlungo_Iptal_Tarihi</x:v>
+        <x:v>Navlungo_Cancelled_At</x:v>
       </x:c>
       <x:c r="Y1" t="str">
-        <x:v>Navlungo_Iptal_Sonucu</x:v>
+        <x:v>Navlungo_Test_Mu</x:v>
       </x:c>
       <x:c r="Z1" t="str">
+        <x:v>Navlungo_Payload_Hash</x:v>
+      </x:c>
+      <x:c r="AA1" t="str">
         <x:v>Kontrol_Uyarısı</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
wire v6.5 navlungo api into apps script runtime
</commit_message>
<xml_diff>
--- a/02_SHEET_SISTEM/Tesbih_Kuyusu_V6_5_Ultra_Operasyon_Sheet.xlsx
+++ b/02_SHEET_SISTEM/Tesbih_Kuyusu_V6_5_Ultra_Operasyon_Sheet.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_WHATSAPP_KUYRUGU" sheetId="1" r:id="R29176c4f133e44f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ACIK_SIPARISLER" sheetId="2" r:id="Rebc28217d49f4356"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_URUN_KALEMLERI" sheetId="3" r:id="Re205233853684fe7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ODEMELER" sheetId="4" r:id="R6c70a1d0f5104a3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_FATURA_GRUPLARI" sheetId="5" r:id="Raff87fc0044041f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_PARASUT_FATURA" sheetId="6" r:id="R1e898b85c7c54496"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_KARGO_PAKETLERI" sheetId="7" r:id="R2beb48ed65444628"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_MUSTERI_HAFIZA" sheetId="8" r:id="Rf4a82754f6b84582"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_808_FINANS_ONIZLEME" sheetId="9" r:id="R35b120c780924ca2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_EBELGE_ISTISNA" sheetId="10" r:id="R9a056e181e0441c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_KONTROL_MERKEZI" sheetId="11" r:id="Re6fef80ec4a64a23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_BANKA_HAREKETLERI" sheetId="12" r:id="R2ba8cbb7154945fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_MUSTERI_ADRESLERI" sheetId="13" r:id="R369895bd379e4fed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_KULLANIM_KILAVUZU" sheetId="14" r:id="Rc0856524bbe04941"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_AYARLAR" sheetId="15" r:id="Rb8d9f5a8cd8744c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_VERI_SOZLUGU" sheetId="16" r:id="R349b5d4496f04817"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_WHATSAPP_KUYRUGU" sheetId="1" r:id="Re9fe5d90bc1b44aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ACIK_SIPARISLER" sheetId="2" r:id="Raa76f48eecb14458"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_URUN_KALEMLERI" sheetId="3" r:id="R1dd38d0ba167429c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ODEMELER" sheetId="4" r:id="R38c0041a6d8649b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_FATURA_GRUPLARI" sheetId="5" r:id="Raae5d49d55b54d10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_PARASUT_FATURA" sheetId="6" r:id="Rfb5df0aae6db436e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_KARGO_PAKETLERI" sheetId="7" r:id="R7063f1b33b824178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_MUSTERI_HAFIZA" sheetId="8" r:id="Rbd66ae6437434854"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_808_FINANS_ONIZLEME" sheetId="9" r:id="Rce76a9514fbe4b87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_EBELGE_ISTISNA" sheetId="10" r:id="R923434332f3c4a0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_KONTROL_MERKEZI" sheetId="11" r:id="R52c8cb3715314c11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_BANKA_HAREKETLERI" sheetId="12" r:id="Rb7f0a9be39c84fb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_MUSTERI_ADRESLERI" sheetId="13" r:id="R9b06989937a24215"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_KULLANIM_KILAVUZU" sheetId="14" r:id="R1d4f696378894817"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_AYARLAR" sheetId="15" r:id="R2bbd764a303e4cb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_VERI_SOZLUGU" sheetId="16" r:id="Re4e212c8a42a4862"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4043,45 +4043,45 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>NAVLUNGO_SENDER_ADDRESS_ID</x:v>
-      </x:c>
-      <x:c r="B10" t="str"/>
+        <x:v>NAVLUNGO_TEST_MODE</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Evet</x:v>
+      </x:c>
       <x:c r="C10" t="str">
-        <x:v>Navlungo kayıtlı gönderici adres ID</x:v>
+        <x:v>Navlungo kargo denemeleri test işaretiyle yürür</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="E10" t="str"/>
-      <x:c r="F10" t="str">
-        <x:v>Script Properties önceliklidir</x:v>
-      </x:c>
+      <x:c r="F10" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>NAVLUNGO_DEFAULT_CARRIER_ID</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>NAVLUNGO_SENDER_ADDRESS_ID</x:v>
+      </x:c>
+      <x:c r="B11" t="str"/>
       <x:c r="C11" t="str">
-        <x:v>Varsayılan Navlungo taşıyıcı ID</x:v>
+        <x:v>Navlungo kayıtlı gönderici adres ID</x:v>
       </x:c>
       <x:c r="D11" t="str">
-        <x:v>Evet</x:v>
+        <x:v>Hayır</x:v>
       </x:c>
       <x:c r="E11" t="str"/>
-      <x:c r="F11" t="str"/>
+      <x:c r="F11" t="str">
+        <x:v>Script Properties önceliklidir</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>NAVLUNGO_DEFAULT_POST_TYPE</x:v>
+        <x:v>NAVLUNGO_DEFAULT_CARRIER_ID</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>Varsayılan Navlungo gönderi tipi</x:v>
+        <x:v>Varsayılan Navlungo taşıyıcı ID</x:v>
       </x:c>
       <x:c r="D12" t="str">
         <x:v>Evet</x:v>
@@ -4091,13 +4091,13 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>NAVLUNGO_DEFAULT_DESI</x:v>
+        <x:v>NAVLUNGO_DEFAULT_POST_TYPE</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>Varsayılan Navlungo desi</x:v>
+        <x:v>Varsayılan Navlungo gönderi tipi</x:v>
       </x:c>
       <x:c r="D13" t="str">
         <x:v>Evet</x:v>
@@ -4107,13 +4107,13 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>NAVLUNGO_DEFAULT_PACKAGE_COUNT</x:v>
+        <x:v>NAVLUNGO_DEFAULT_DESI</x:v>
       </x:c>
       <x:c r="B14" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>Varsayılan Navlungo paket adedi</x:v>
+        <x:v>Varsayılan Navlungo desi</x:v>
       </x:c>
       <x:c r="D14" t="str">
         <x:v>Evet</x:v>
@@ -4123,45 +4123,47 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>NAVLUNGO_CARRIER_ID_MAP_JSON</x:v>
+        <x:v>NAVLUNGO_DEFAULT_PACKAGE_COUNT</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>{}</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>Kargo firması -&gt; Navlungo carrier_id map JSON</x:v>
+        <x:v>Varsayılan Navlungo paket adedi</x:v>
       </x:c>
       <x:c r="D15" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="E15" t="str"/>
       <x:c r="F15" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>SISTEM_OPERASYON_SAATI_KAPANIS</x:v>
+        <x:v>NAVLUNGO_CARRIER_ID_MAP_JSON</x:v>
       </x:c>
       <x:c r="B16" t="str">
-        <x:v>16:00</x:v>
+        <x:v>{"Aras Kargo":"1","Yurtiçi Kargo":"2"}</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>Operasyon kapanış saati</x:v>
+        <x:v>Kargo firması -&gt; Navlungo carrier_id map JSON</x:v>
       </x:c>
       <x:c r="D16" t="str">
         <x:v>Evet</x:v>
       </x:c>
       <x:c r="E16" t="str"/>
-      <x:c r="F16" t="str"/>
+      <x:c r="F16" t="str">
+        <x:v>Kargo firması varsa map eşleşmesi zorunludur</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>TCKN_VARSAYILAN_GERCEK_KISI</x:v>
+        <x:v>SISTEM_OPERASYON_SAATI_KAPANIS</x:v>
       </x:c>
       <x:c r="B17" t="str">
-        <x:v>11111111111</x:v>
+        <x:v>16:00</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>Gerçek kişi TCKN boşsa uygulanabilir</x:v>
+        <x:v>Operasyon kapanış saati</x:v>
       </x:c>
       <x:c r="D17" t="str">
         <x:v>Evet</x:v>
@@ -4171,13 +4173,13 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>BANKA_HAREKET_MODULU_AKTIF</x:v>
+        <x:v>TCKN_VARSAYILAN_GERCEK_KISI</x:v>
       </x:c>
       <x:c r="B18" t="str">
-        <x:v>Evet</x:v>
+        <x:v>11111111111</x:v>
       </x:c>
       <x:c r="C18" t="str">
-        <x:v>14 banka hareketi teyit katmanı</x:v>
+        <x:v>Gerçek kişi TCKN boşsa uygulanabilir</x:v>
       </x:c>
       <x:c r="D18" t="str">
         <x:v>Evet</x:v>
@@ -4187,35 +4189,51 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>VARSAYILAN_KARGO_FIRMASI</x:v>
+        <x:v>BANKA_HAREKET_MODULU_AKTIF</x:v>
       </x:c>
       <x:c r="B19" t="str">
-        <x:v>Aras Kargo</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>Kargo firması önerisi</x:v>
+        <x:v>14 banka hareketi teyit katmanı</x:v>
       </x:c>
       <x:c r="D19" t="str">
-        <x:v>Hayır</x:v>
+        <x:v>Evet</x:v>
       </x:c>
       <x:c r="E19" t="str"/>
       <x:c r="F19" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
-        <x:v>KARGO_UCRETI_STANDART</x:v>
+        <x:v>VARSAYILAN_KARGO_FIRMASI</x:v>
       </x:c>
       <x:c r="B20" t="str">
-        <x:v>125</x:v>
+        <x:v>Aras Kargo</x:v>
       </x:c>
       <x:c r="C20" t="str">
-        <x:v>808 finans ön izleme için varsayılan maliyet</x:v>
+        <x:v>Kargo firması önerisi</x:v>
       </x:c>
       <x:c r="D20" t="str">
         <x:v>Hayır</x:v>
       </x:c>
       <x:c r="E20" t="str"/>
       <x:c r="F20" t="str"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>KARGO_UCRETI_STANDART</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>808 finans ön izleme için varsayılan maliyet</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>Hayır</x:v>
+      </x:c>
+      <x:c r="E21" t="str"/>
+      <x:c r="F21" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>